<commit_message>
Add auth suites: order history (A7), forget-password (A4), tab switch
New Robot Framework tests (verified green on staging, today=2026-06-30):
- tests/auth/user/TC-OH-02   order history empty state ("- ยังไม่มีรายการสั่งซื้อ -")
- tests/auth/user/TC-USER-13 user-infos tab switch (ข้อมูลส่วนตัว <-> รายการสั่งซื้อ)
- tests/auth/forget/TC-FGT-01 reset link sent for a registered email
- tests/auth/forget/TC-FGT-03 unknown email -> backend error (no client validation;
  also covers TC-FGT-02's error message without a mock)

Supporting:
- auth keywords/locators: orders tab, forget-password page + Request Password Reset
- routes: USER_INFOS, FORGET_PASSWORD
- tracker xlsx: statuses updated; TC-OH-01/03/04 Blocked (need a user with orders, TD-39);
  TC-FGT-04 Blocked (FINDING: loading button not actually disabled).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -7837,10 +7837,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -7849,7 +7845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11 เคส (ดูคอลัมน์ Script File ของแต่ละเคส)</t>
+          <t>15 เคส (เพิ่ม TC-FGT-01 reset link, TC-FGT-03 invalid email)</t>
         </is>
       </c>
     </row>
@@ -7885,13 +7881,9 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TC-USER-01 guest gate / 02 prefill / 05 email read-only / 12 logout</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
+          <t>TC-USER-01 guest / 02 prefill / 05 email RO / 12 logout / 13 tab switch ; TC-OH-02 empty orders</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -7953,10 +7945,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-    </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -7970,7 +7958,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>- เพิ่ม helper first-visible input/click + retry กัน stale element</t>
@@ -7978,7 +7965,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>- เพิ่ม keyword ปฏิทินจัดส่ง (boundary) + coupon apply/error</t>
@@ -7986,7 +7972,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>- เพิ่ม date helper relative_aria_label / aria_date_part</t>
@@ -7994,16 +7979,11 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>- coupons.json ใส่ code staging จริง; route USER_INFOS</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -8018,7 +7998,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t xml:space="preserve">  --pythonpath libraries --pythonpath . \</t>
@@ -8026,7 +8005,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t xml:space="preserve">  --variablefile resources/variables/env_staging.yaml \</t>
@@ -8034,16 +8012,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t xml:space="preserve">  --exclude createsorder --outputdir results tests</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -10498,7 +10471,7 @@
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I28" s="9" t="inlineStr">
@@ -10507,7 +10480,11 @@
         </is>
       </c>
       <c r="J28" s="9" t="n"/>
-      <c r="K28" s="9" t="n"/>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>tests/auth/forget/TC-FGT-01_send-reset-link-success.robot — PASS (ส่งอีเมลจริงไป TD-30)</t>
+        </is>
+      </c>
       <c r="L28" s="9" t="inlineStr">
         <is>
           <t>TD-30</t>
@@ -10573,7 +10550,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
@@ -10582,7 +10559,11 @@
         </is>
       </c>
       <c r="J29" s="9" t="n"/>
-      <c r="K29" s="9" t="n"/>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>error message ครอบโดย TC-FGT-03 แล้ว; การ mock 500 จริงรอ API track (RequestsLibrary/CDP)</t>
+        </is>
+      </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
           <t>mock 500</t>
@@ -10648,7 +10629,7 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I30" s="9" t="inlineStr">
@@ -10657,7 +10638,11 @@
         </is>
       </c>
       <c r="J30" s="9" t="n"/>
-      <c r="K30" s="9" t="n"/>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>tests/auth/forget/TC-FGT-03_invalid-email-error.robot — PASS (ครอบ error ของ FGT-02 ด้วย)</t>
+        </is>
+      </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -10719,16 +10704,20 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J31" s="9" t="n"/>
-      <c r="K31" s="9" t="n"/>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>FINDING: ปุ่มเปลี่ยน text เป็น "กำลังดำเนินการ" แต่ disabled=false (ไม่ได้กันกดซ้ำจริง) — ยืนยันกับ dev</t>
+        </is>
+      </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
           <t>TD-30</t>
@@ -12085,7 +12074,7 @@
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I49" s="9" t="inlineStr">
@@ -12094,7 +12083,11 @@
         </is>
       </c>
       <c r="J49" s="9" t="n"/>
-      <c r="K49" s="9" t="n"/>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>tests/auth/user/TC-USER-13_tab-switch.robot — PASS</t>
+        </is>
+      </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
           <t>TD-30</t>
@@ -12160,7 +12153,7 @@
       </c>
       <c r="H50" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I50" s="9" t="inlineStr">
@@ -12169,7 +12162,11 @@
         </is>
       </c>
       <c r="J50" s="9" t="n"/>
-      <c r="K50" s="9" t="n"/>
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>รอ user ที่มีออเดอร์ (TD-39) จาก dev</t>
+        </is>
+      </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
           <t>TD-39</t>
@@ -12235,7 +12232,7 @@
       </c>
       <c r="H51" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I51" s="9" t="inlineStr">
@@ -12244,7 +12241,11 @@
         </is>
       </c>
       <c r="J51" s="9" t="n"/>
-      <c r="K51" s="9" t="n"/>
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>tests/auth/user/TC-OH-02_order-history-empty.robot — PASS (inoobeam ไม่มีออเดอร์)</t>
+        </is>
+      </c>
       <c r="L51" s="9" t="inlineStr">
         <is>
           <t>user ไม่มีออเดอร์</t>
@@ -12310,7 +12311,7 @@
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I52" s="9" t="inlineStr">
@@ -12319,7 +12320,11 @@
         </is>
       </c>
       <c r="J52" s="9" t="n"/>
-      <c r="K52" s="9" t="n"/>
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>copy order code — รอ user ที่มีออเดอร์ (TD-39)</t>
+        </is>
+      </c>
       <c r="L52" s="9" t="inlineStr">
         <is>
           <t>TD-39</t>
@@ -12385,7 +12390,7 @@
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I53" s="9" t="inlineStr">
@@ -12394,7 +12399,11 @@
         </is>
       </c>
       <c r="J53" s="9" t="n"/>
-      <c r="K53" s="9" t="n"/>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>LINE link — รอ user ที่มีออเดอร์ (TD-39)</t>
+        </is>
+      </c>
       <c r="L53" s="9" t="inlineStr">
         <is>
           <t>TD-39</t>

</xml_diff>

<commit_message>
Add Product Discovery suite (TC-DISC-04/09/10)
New Robot Framework tests (verified green on staging):
- tests/discovery/TC-DISC-04  pagination: 15/page + ?page=2 kept in URL
- tests/discovery/TC-DISC-09  express + promotion listings render with products
- tests/discovery/TC-DISC-10  near-me (wreath-nearme) listing renders

Supporting:
- category keywords: Get Listing Card Count, Go To Next Listing Page (waits for SPA
  async ?page= update), Assert Page Is Not 404 (retries past transient flash).
- locator CAT_NEXT_PAGE; categories.json: near_me, donate.

Findings recorded in tracker (Blocked):
- TC-DISC-01 sort not reflected in URL (only ?page=1, order unchanged)
- TC-DISC-03 ?keyword= does not filter results
- /wreath-donate flashes "ไม่พบหน้า" when empty (donate smoke dropped)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -7845,7 +7845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15 เคส (เพิ่ม TC-FGT-01 reset link, TC-FGT-03 invalid email)</t>
+          <t>18 เคส (+ Product Discovery: DISC-04 pagination, DISC-09 listings, DISC-10 near-me)</t>
         </is>
       </c>
     </row>
@@ -13613,16 +13613,20 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>FINDING: เลือก sort แล้ว URL ได้แค่ ?page=1 ไม่มี sort= และลำดับไม่เปลี่ยน — ยืนยันกับ dev</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>listing</t>
@@ -13763,16 +13767,20 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>?keyword=บุหลัน ไม่กรองผล (15 เท่าเดิม) — ยืนยัน behavior กับ dev</t>
+        </is>
+      </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -13838,7 +13846,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -13847,7 +13855,11 @@
         </is>
       </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>tests/discovery/TC-DISC-04_pagination.robot — PASS (15/หน้า, ?page=2)</t>
+        </is>
+      </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
           <t>listing &gt;15 ชิ้น</t>
@@ -14213,7 +14225,7 @@
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
@@ -14222,7 +14234,11 @@
         </is>
       </c>
       <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>tests/discovery/TC-DISC-09_special-listings-smoke.robot — PASS (express+promotion); donate ตัดออก (finding)</t>
+        </is>
+      </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -14284,7 +14300,7 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
@@ -14293,7 +14309,11 @@
         </is>
       </c>
       <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>tests/discovery/TC-DISC-10_near-me-smoke.robot — PASS</t>
+        </is>
+      </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Complete Product Discovery suite (TC-DISC-05/08)
- tests/discovery/TC-DISC-08  promotion product shows struck regular price (H014 ฿1,899)
- tests/discovery/TC-DISC-05  wizard listing (products-special) renders (smoke)
- product keyword Assert Promotion Price Shown; categories.json wizard_special

Remaining F cases recorded Blocked in tracker with findings:
- TC-DISC-02 filter not standard checkboxes / likely not URL-reflected
- TC-DISC-06 needs a confirmed EXCLUDED_TAGS slug
- TC-DISC-07 testdata not-orderable slug still shows buy buttons (need TD-04)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -7845,7 +7845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>18 เคส (+ Product Discovery: DISC-04 pagination, DISC-09 listings, DISC-10 near-me)</t>
+          <t>20 เคส (Product Discovery: DISC-04/05/08/09/10)</t>
         </is>
       </c>
     </row>
@@ -13692,16 +13692,20 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>filter ไม่ใช่ checkbox มาตรฐาน/ซ่อน + คาดว่าไม่ reflect URL (เทียบ sort) — ต้อง probe ลึก</t>
+        </is>
+      </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>listing</t>
@@ -13925,16 +13929,20 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>tests/discovery/TC-DISC-05_wizard-listing-smoke.robot — PASS (smoke; cookie-match รอ TD-37)</t>
+        </is>
+      </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
           <t>TD-37</t>
@@ -14000,16 +14008,20 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>ต้องมี slug สินค้าที่ติด EXCLUDED_TAGS ที่ยืนยันแล้ว เพื่อ assert ว่าไม่โผล่</t>
+        </is>
+      </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
           <t>หมวดมี excluded tag</t>
@@ -14075,7 +14087,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -14084,7 +14096,11 @@
         </is>
       </c>
       <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>testdata slug b301-wnw-วลิลา-01-16 ยังมีปุ่มซื้อ (ไม่ใช่ allow_add_to_cart=false) — รอ slug จริง TD-04</t>
+        </is>
+      </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
           <t>TD-04</t>
@@ -14150,7 +14166,7 @@
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
@@ -14159,7 +14175,11 @@
         </is>
       </c>
       <c r="J9" s="9" t="n"/>
-      <c r="K9" s="9" t="n"/>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>tests/discovery/TC-DISC-08_promotion-price.robot — PASS (H014 ราคาตัดทอน ฿1,899)</t>
+        </is>
+      </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
           <t>สินค้ามีโปร</t>

</xml_diff>

<commit_message>
Add Global components suite (TC-GBL-02/04)
- tests/global/TC-GBL-02  header cart badge reflects item count
- tests/global/TC-GBL-04  back-to-top button scrolls page to top
- locator BACK_TO_TOP_BTN (icon-only fixed button)

GBL-01/03/05 marked Skipped in tracker (weak/ambiguous hooks: announcement close
tied to cookie ×, mobile floating/sticky, hamburger has no stable selector).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -7845,7 +7845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20 เคส (Product Discovery: DISC-04/05/08/09/10)</t>
+          <t>22 เคส (+ Global: GBL-02 cart badge, GBL-04 back-to-top)</t>
         </is>
       </c>
     </row>
@@ -16666,16 +16666,20 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>announcement bar = strip "ส่งฟรีทั่ว กทม." แสดงได้ แต่ปุ่มปิดผูกกับ cookie × คลุมเครือ — เลื่อนไว้</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>มี announcement active</t>
@@ -16737,16 +16741,20 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>tests/global/TC-GBL-02_minicart-badge.robot — PASS (badge=1; dropdown ไม่ assert)</t>
+        </is>
+      </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>มีของในตะกร้า</t>
@@ -16812,16 +16820,20 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>floating contact/sticky (mobile) — hook อ่อน ต้อง probe viewport เพิ่ม</t>
+        </is>
+      </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>mobile</t>
@@ -16883,7 +16895,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -16892,7 +16904,11 @@
         </is>
       </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>tests/global/TC-GBL-04_back-to-top.robot — PASS (ปุ่ม fixed bottom-20)</t>
+        </is>
+      </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
           <t>หน้ายาว</t>
@@ -16954,16 +16970,20 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>hamburger/MobileNavBar — ยังไม่เจอ selector ชัด (ไม่มี aria/class ตรง) ต้อง probe เพิ่ม</t>
+        </is>
+      </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
           <t>mobile viewport</t>

</xml_diff>

<commit_message>
Add Content/SEO smoke suite (TC-CMS-04/05/07)
- tests/content/TC-CMS-05  8 info pages load with title + canonical (faqs, contact,
  policies, how-to-order, about-us, flower-shop, review-wreath)
- tests/content/TC-CMS-04  service-funeral + all-service load (SEO smoke)
- tests/content/TC-CMS-07  unknown slug shows NotfoundPage
- common keyword Assert Content Page Loads + Not Found Marker Should Be Hidden/Visible
  (404 check uses VISIBLE innerText — NotFound markup ships in every page's HTML, so a
  page-source check false-passes/false-fails)

Findings/Blocked in tracker:
- service-crematory/-pet/-relics return 404 (route slugs don't match doc)
- TC-CMS-01/02/03 (articles/author) need real slugs (TD-38)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -7845,7 +7845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>22 เคส (+ Global: GBL-02 cart badge, GBL-04 back-to-top)</t>
+          <t>25 เคส (+ Content/SEO: CMS-04 service, CMS-05 info×8, CMS-07 404)</t>
         </is>
       </c>
     </row>
@@ -14517,7 +14517,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
@@ -14526,7 +14526,11 @@
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>บทความ listing/filter — รอ article slug จริง (TD-38)</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>TD-38</t>
@@ -14592,7 +14596,7 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
@@ -14601,7 +14605,11 @@
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>บทความ detail — รอ slug (TD-38)</t>
+        </is>
+      </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>TD-38</t>
@@ -14667,7 +14675,7 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
@@ -14676,7 +14684,11 @@
         </is>
       </c>
       <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>ผู้เขียน — รอ author slug (TD-38)</t>
+        </is>
+      </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>TD-38</t>
@@ -14742,7 +14754,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -14751,7 +14763,11 @@
         </is>
       </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>tests/content/TC-CMS-04_service-pages-smoke.robot — PASS (funeral+all-service); crematory/pet/relics → 404 (finding route ไม่ตรง)</t>
+        </is>
+      </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -14813,16 +14829,20 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>tests/content/TC-CMS-05_info-pages-smoke.robot — PASS 8 หน้า (title+canonical)</t>
+        </is>
+      </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -14955,7 +14975,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -14964,7 +14984,11 @@
         </is>
       </c>
       <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>tests/content/TC-CMS-07_unknown-slug-404.robot — PASS (เช็ค visible text; NotFound markup ติดมาใน HTML ทุกหน้า)</t>
+        </is>
+      </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Add Message Card validation test (TC-CARD-03)
- tests/messagecard/TC-CARD-03  line-1 empty -> save ("ตกลง") disabled + required hint
- checkout keywords Open Ribbon Modal, Assert Ribbon Save Disabled
- MSG_CARD_LINE1_REQUIRED

Tracker: TC-CARD-05 marked done (covered by TC-CHK-13). CARD-01/02/04/10 Blocked
(message-card preview/base64 does not render under headless Selenium, so save never
enables in-test); CARD-06/07/08 Blocked (need logo image fixtures / media mock).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -7845,7 +7845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>25 เคส (+ Content/SEO: CMS-04 service, CMS-05 info×8, CMS-07 404)</t>
+          <t>26 เคส (+ Message Card: CARD-03 line1 required)</t>
         </is>
       </c>
     </row>
@@ -12591,16 +12591,20 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>preview base64 ไม่ render ใน headless (888ms debounce/ API) — save ไม่ enable ภายใน 3s</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>สินค้าใน checkout</t>
@@ -12666,16 +12670,20 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>tone/format/align preview — ขึ้นกับ preview render (ดู CARD-01)</t>
+        </is>
+      </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>เปิด modal</t>
@@ -12741,7 +12749,7 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
@@ -12750,7 +12758,11 @@
         </is>
       </c>
       <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>tests/messagecard/TC-CARD-03_line1-required.robot — PASS (save disabled + กรุณาระบุ "ข้อความบรรทัดที่ 1")</t>
+        </is>
+      </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>เปิด modal</t>
@@ -12816,16 +12828,20 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>บันทึก→card-final ต้องรอ preview/finalId (render ช้าใน headless)</t>
+        </is>
+      </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
           <t>กรอกบรรทัด 1</t>
@@ -12891,7 +12907,7 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
@@ -12900,7 +12916,11 @@
         </is>
       </c>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>ครอบโดย tests/checkout_rules/TC-CHK-13_message-card-count.robot (2 พวง กรอก 1 → submit disable)</t>
+        </is>
+      </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
           <t>TD-36 (2 พวง)</t>
@@ -12966,16 +12986,20 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>logo ใหญ่เกิน — ต้องไฟล์รูป &gt;288px (TD-35)</t>
+        </is>
+      </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
           <t>TD-35 รูปใหญ่</t>
@@ -13041,7 +13065,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -13050,7 +13074,11 @@
         </is>
       </c>
       <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>อัปโหลดล้มเหลว — ต้อง mock media API</t>
+        </is>
+      </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
           <t>mock media error</t>
@@ -13116,16 +13144,20 @@
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J9" s="9" t="n"/>
-      <c r="K9" s="9" t="n"/>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>ไฟล์ non-image — ต้องไฟล์ตัวอย่าง (TD-35)</t>
+        </is>
+      </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
           <t>TD-35 non-image</t>
@@ -13266,16 +13298,20 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>cleanup localStorage — ต้องบันทึกป้ายได้ก่อน (ติด CARD-04)</t>
+        </is>
+      </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
           <t>มีป้าย+สินค้า</t>

</xml_diff>

<commit_message>
Update tracker: cumulative progress tally (2026-06-30)
Add a static project-wide tally to the Progress sheet (per-sheet + grand total),
so totals are readable without Excel recomputing the COUNTIF summaries.

Snapshot: Script Done 65/188 (35%), Blocked 28, Skipped 3, Not Started 92.
This session added 26 new automated cases (Coupon, Checkout rules, Auth, Product
Discovery, Global, Content/SEO, Message Card).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -40,7 +40,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="12">
@@ -159,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +206,7 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7818,11 +7823,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8039,6 +8048,301 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>repo file checkout/TC-CHK-09_out-of-province ใช้ ID ผิด (ที่จริง=TC-CART-05-R)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>── ยอดสะสมทั้งโปรเจกต์ (อัปเดต 2026-06-30) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Sheet / โมดูล</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>checkout</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>75</v>
+      </c>
+      <c r="C30" t="n">
+        <v>25</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>A-Account-Auth</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>52</v>
+      </c>
+      <c r="C31" t="n">
+        <v>28</v>
+      </c>
+      <c r="D31" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>B-MessageCard</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>7</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>F-ProductDiscovery</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>10</v>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>G-Content-SEO</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>H-LINE-B2B</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>I-Tracking</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>6</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>J-Contact-Corporate</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>K-Global</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>L-Cross-cutting</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>รวมทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>188</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Script Done = 65/188 (35%)  ·  ไฟล์ .robot จริง = 93</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ทำใน session นี้ (ใหม่) = 26 เคส: Coupon4 · CHK-rules3 · Auth7 · Discovery5 · Global2 · Content11(*) · MsgCard2  (* CMS-05 นับ 8 หน้าเป็น 1 TC)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Open API track: api_library + TC-API-01; record /api/order 500 bug
- libraries/api_library.py — thin requests wrapper (RequestsLibrary not installed):
  API Post Json / API Get returning {status, json, text}
- tests/api/TC-API-01 — POST /api/order {} → 422 {error:true} structured (proxy error
  path, no browser, no order created). Also covers TC-XAPI-01.
- tests/api/TC-CHK-12 — Skip(BLOCKED): backend returns 500 "Undefined array key count"
  (OrderController.php:176) for an unknown-slug cart instead of a 422 slug-rule rejection.
- dev request doc §3.8 records the 500 bug; tracker updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -3318,13 +3318,13 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>API-level: POST /api/order payload — รอเปิด RequestsLibrary</t>
+          <t>tests/api/TC-CHK-12 (skip): backend 500 "Undefined array key count" แทน 422 slug-rule — bug §3.8 รอ dev</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -6128,12 +6128,20 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr"/>
+          <t>Script Done</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J71" s="2" t="inlineStr"/>
-      <c r="K71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>tests/api/TC-API-01_order-empty-payload-422.robot — PASS (POST /api/order {} → 422 error:true) via api_library</t>
+        </is>
+      </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
           <t>mock ERP 422 (TD-24)</t>
@@ -6716,16 +6724,20 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>ครอบโดย tests/api/TC-API-01 (POST /api/order {} → 422 error:true ไม่ crash)</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>mock 422</t>
@@ -7845,7 +7857,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>26 เคส (+ Message Card: CARD-03 line1 required)</t>
+          <t>27 เคส + เปิด API track (TC-API-01 ผ่าน; TC-CHK-12 พบ bug 500)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 9 no-data tests (sitemap, contact/corporate, LINE cookie routes) — all green
- TC-CMS-08 sitemap XML; TC-CT-01/02/03 contact + corporate (channels/FAQ/gallery)
- TC-LINE-01/02/04/05/06 landing routes set distinct cookies (user_id/_b2b/_event)
  and coexist; TC-LINE-03 (external openline redirect) deferred
- New keywords: Assert Sitemap Xml, Page Should Have Link To, Assert Image Count
  At Least, Open Route And Settle, Cookie Should Be Set
- xlsx: mark 16 cases Script Done (this session) — 83/188 (44%)

Verified live on staging 2026-07-02.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -1654,12 +1654,16 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>tests/product/TC-PDP-05_non-orderable.robot — live PASS 2026-07-02 (d040 ซ่อนปุ่มซื้อ + LINE)</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>TD-04</t>
@@ -3708,7 +3712,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3719,7 +3723,7 @@
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>รอ valid code ที่ loginUser ยังไม่เคยใช้ (QA-Coupon-TestData-Request.md §1.1)</t>
+          <t>tests/promo/TC-PROMO-01-R_valid-coupon-applies-discount.robot — live PASS 2026-07-02 (validate-only/reusable, คูปอง 10%)</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -4040,7 +4044,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -4051,7 +4055,7 @@
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>ยอด&lt;min ทำไม่ได้ (สินค้าถูกสุด ~1,599 &gt; min 1,000) — รอ data</t>
+          <t>tests/promo/TC-PROMO-05_below-min-not-applied.robot — live PASS 2026-07-02 (ตะกร้า ฿1599 &lt; min ฿2000 → ไม่หัก)</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -8726,7 +8730,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -8737,7 +8741,7 @@
       <c r="J5" s="9" t="n"/>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>tests/auth/login/TC-LOGIN-04_unverified-email.robot</t>
+          <t>tests/auth/login/TC-LOGIN-04_unverified-email.robot — live PASS 2026-07-02 (unverified user)</t>
         </is>
       </c>
       <c r="L5" s="9" t="inlineStr">
@@ -14135,7 +14139,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -14146,7 +14150,7 @@
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>testdata slug b301-wnw-วลิลา-01-16 ยังมีปุ่มซื้อ (ไม่ใช่ allow_add_to_cart=false) — รอ slug จริง TD-04</t>
+          <t>tests/discovery/TC-DISC-07_non-orderable-line.robot — live PASS 2026-07-02 (d040)</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
@@ -14565,7 +14569,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
@@ -14576,7 +14580,7 @@
       <c r="J2" s="9" t="n"/>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>บทความ listing/filter — รอ article slug จริง (TD-38)</t>
+          <t>tests/content/TC-CMS-01_article-listing-smoke.robot — live PASS 2026-07-02</t>
         </is>
       </c>
       <c r="L2" s="9" t="inlineStr">
@@ -14644,7 +14648,7 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
@@ -14655,7 +14659,7 @@
       <c r="J3" s="9" t="n"/>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>บทความ detail — รอ slug (TD-38)</t>
+          <t>tests/content/TC-CMS-02_article-detail-jsonld.robot — live PASS 2026-07-02 (+JSON-LD)</t>
         </is>
       </c>
       <c r="L3" s="9" t="inlineStr">
@@ -15098,7 +15102,7 @@
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
@@ -15107,7 +15111,11 @@
         </is>
       </c>
       <c r="J9" s="9" t="n"/>
-      <c r="K9" s="9" t="n"/>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>tests/content/TC-CMS-08_sitemap.robot — live PASS 2026-07-02</t>
+        </is>
+      </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -15291,7 +15299,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
@@ -15300,7 +15308,11 @@
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>tests/line/TC-LINE_cookie-routes.robot — live PASS 2026-07-02</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>clear cookie</t>
@@ -15362,7 +15374,7 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
@@ -15371,7 +15383,11 @@
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>tests/line/TC-LINE_cookie-routes.robot — live PASS 2026-07-02 (persist)</t>
+        </is>
+      </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>มี cookie</t>
@@ -15504,7 +15520,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -15513,7 +15529,11 @@
         </is>
       </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>tests/line/TC-LINE_cookie-routes.robot — live PASS 2026-07-02 (user_id_b2b)</t>
+        </is>
+      </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -15575,7 +15595,7 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
@@ -15584,7 +15604,11 @@
         </is>
       </c>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>tests/line/TC-LINE_cookie-routes.robot — live PASS 2026-07-02 (user_id_event)</t>
+        </is>
+      </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -15646,7 +15670,7 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
@@ -15655,7 +15679,11 @@
         </is>
       </c>
       <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>tests/line/TC-LINE_cookie-routes.robot — live PASS 2026-07-02 (3 cookies distinct)</t>
+        </is>
+      </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -16403,7 +16431,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
@@ -16412,7 +16440,11 @@
         </is>
       </c>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>tests/contact/TC-CT-01_contact-channels.robot — live PASS 2026-07-02 (LINE/tel/email)</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -16474,7 +16506,7 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
@@ -16483,7 +16515,11 @@
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>tests/contact/TC-CT-02_corporate-faq.robot — live PASS 2026-07-02 (FAQ + credit/invoice)</t>
+        </is>
+      </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -16545,7 +16581,7 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
@@ -16554,7 +16590,11 @@
         </is>
       </c>
       <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>tests/contact/TC-CT-03_corporate-contact-gallery.robot — live PASS 2026-07-02 (lineb2b/tel/gallery)</t>
+        </is>
+      </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Add TC-TRK2-04 (invalid tracking id, no leak) + TC-CMS-06 (dynamic Thai router)
Both verified live on staging 2026-07-02. xlsx marked Script Done — 85/188 (45%).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -14956,7 +14956,7 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
@@ -14965,7 +14965,11 @@
         </is>
       </c>
       <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>tests/content/TC-CMS-06_dynamic-router.robot — live PASS 2026-07-02 (4 Thai slugs)</t>
+        </is>
+      </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -16092,7 +16096,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -16101,7 +16105,11 @@
         </is>
       </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>tests/tracking/TC-TRK2-04_invalid-tracking-id-no-leak.robot — live PASS 2026-07-02</t>
+        </is>
+      </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Add checkout FE validation gate tests (TC-CHK-02-R/03/04-UI) — all green
Empty required fields, invalid email, and invalid phone each keep the
"ชำระเงิน" submit button disabled (FE validation gate). Reuses Fill Delivery
And Buyer + Assert Submit Disabled. Verified live on staging 2026-07-02.
xlsx → 88/188 (47%).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -2456,12 +2456,16 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>tests/checkout/TC-CHK-02-R_required-fields-gate.robot — live PASS 2026-07-02 (submit disabled)</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
           <t>กรอกเกือบครบ</t>
@@ -2531,12 +2535,16 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>tests/checkout/TC-CHK-03_invalid-email-gate.robot — live PASS 2026-07-02 (bad email → gated)</t>
+        </is>
+      </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
           <t>อยู่ checkout</t>
@@ -2606,12 +2614,16 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>tests/checkout/TC-CHK-04-UI_invalid-phone-gate.robot — live PASS 2026-07-02 (bad phone → gated)</t>
+        </is>
+      </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
           <t>อยู่ checkout</t>

</xml_diff>

<commit_message>
Add SEO/cart green tests: TC-XPERF-02, TC-CART-03-R, TC-CHK-06-R — all green
- TC-XPERF-02 PDP canonical + Open Graph + JSON-LD
- TC-CART-03-R guest cart persists across reload
- TC-CHK-06-R grand total sums two distinct items (1599+2899=4498)
New keywords: Assert JsonLd Present, Assert Open Graph Present.
Verified live 2026-07-02. xlsx → 91/188 (48%).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -1982,12 +1982,16 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/TC-CART-03-R_guest-cart-persist.robot — live PASS 2026-07-02</t>
+        </is>
+      </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
           <t>guest, มีสินค้า</t>
@@ -2847,12 +2851,16 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>tests/checkout/TC-CHK-06-R_multi-item-total.robot — live PASS 2026-07-02 (1599+2899=4498)</t>
+        </is>
+      </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
           <t>2-3 สินค้า, login (ถ้าใช้คูปอง)</t>
@@ -7415,7 +7423,7 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
@@ -7424,7 +7432,11 @@
         </is>
       </c>
       <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>tests/global/TC-XPERF-02_seo-structured-data.robot — live PASS 2026-07-02 (canonical/og/JSON-LD)</t>
+        </is>
+      </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Add TC-HOME-02 (home social/contact links smoke) — green
Home exposes LINE (/line/), tel: and facebook links. Verified live 2026-07-02.
xlsx → 92/188 (49%).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -797,12 +797,16 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Script Done</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>tests/home/TC-HOME-02_social-contact-links.robot — live PASS 2026-07-02</t>
+        </is>
+      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Home โหลดสำเร็จ</t>

</xml_diff>

<commit_message>
Mark payment/2C2P/order-success cases as Skipped (manual, no sandbox)
10 cases require a real order + 2C2P sandbox (dev: not supported) → manual test,
out of automation scope: TC-PAY-01-R/02-R/03/04/05/06/07/09, TC-ORD-01a-R/01b-R.
Automation coverage now 92/175 automatable (53%).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
+++ b/docs/QA-WreathNaWat-Checkout-OrderFlow-TestCases.xlsx
@@ -4783,12 +4783,16 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr"/>
-      <c r="K53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
           <t>order รอชำระ (TD-20)</t>
@@ -4858,12 +4862,16 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
           <t>ผ่าน checkout, ยอดทราบค่า (TD-18)</t>
@@ -4933,12 +4941,16 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="inlineStr"/>
-      <c r="K55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
           <t>อยู่หน้าชำระเงิน</t>
@@ -5008,12 +5020,16 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
-      <c r="K56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
           <t>ผ่าน checkout (TD-18)</t>
@@ -5083,12 +5099,16 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr"/>
-      <c r="K57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
           <t>order รอชำระ (TD-20)</t>
@@ -5158,12 +5178,16 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="inlineStr"/>
-      <c r="K58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
           <t>order รอชำระ</t>
@@ -5233,12 +5257,16 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
           <t>order รอชำระ</t>
@@ -5308,12 +5336,16 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
           <t>order รอชำระ</t>
@@ -5466,12 +5498,16 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
           <t>order สำเร็จ (sandbox)</t>
@@ -5541,12 +5577,16 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Manual (ไม่มี 2C2P sandbox / ต้องสร้าง order+ชำระเงินจริง) — ตัดออกจาก automation scope</t>
+        </is>
+      </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
           <t>order สำเร็จ</t>

</xml_diff>